<commit_message>
template update for business and agent stf bulk
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/organisation/stf/STF organisation - One valid row.xlsx
+++ b/src/test/resources/testData/organisation/stf/STF organisation - One valid row.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/karthik.jaladurgam/Desktop/STOS/Test data/Business/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A88F32A8-49CB-714C-8506-18A55DF575CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8091AAA4-DBAD-B242-BA33-44BD3F8E3B6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17580" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -313,7 +313,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -333,13 +333,6 @@
       <name val="Aptos Narrow"/>
     </font>
     <font>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <u/>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Arial"/>
@@ -401,7 +394,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -417,9 +410,6 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -685,7 +675,7 @@
       <c r="K1" t="s">
         <v>44</v>
       </c>
-      <c r="L1" s="9" t="s">
+      <c r="L1" s="8" t="s">
         <v>65</v>
       </c>
       <c r="M1" t="s">
@@ -836,7 +826,7 @@
       <c r="K3" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="L3" s="7" t="s">
+      <c r="L3" s="6" t="s">
         <v>27</v>
       </c>
       <c r="M3" s="5"/>
@@ -923,7 +913,7 @@
       <c r="N4" s="5">
         <v>12345678</v>
       </c>
-      <c r="O4" s="8">
+      <c r="O4" s="7">
         <v>46023</v>
       </c>
       <c r="P4" s="5" t="s">
@@ -967,7 +957,7 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="L3" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="L3" r:id="rId1" xr:uid="{084FA068-A3C3-7D41-BBD1-F3839A98D4FD}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>

</xml_diff>